<commit_message>
update salary slip template
</commit_message>
<xml_diff>
--- a/salaryData/test12.xlsx
+++ b/salaryData/test12.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MERCURY\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MERCURY\Desktop\lanatus\projects\business-automation\salaryData\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <si>
     <t>jimit</t>
   </si>
@@ -44,18 +44,9 @@
     <t>HRA</t>
   </si>
   <si>
-    <t>piyushk@lanatussystems.com</t>
-  </si>
-  <si>
-    <t>piyush</t>
-  </si>
-  <si>
     <t>jimitm@lanatussystems.com</t>
   </si>
   <si>
-    <t>Full stack developer</t>
-  </si>
-  <si>
     <t>Bank_Account_Number</t>
   </si>
   <si>
@@ -80,26 +71,83 @@
     <t>Payslip_For_The_Month</t>
   </si>
   <si>
-    <t>Basic_Salary</t>
-  </si>
-  <si>
     <t>Other_Allowances</t>
   </si>
   <si>
-    <t>Total_Earnings</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 07-03-2022</t>
   </si>
   <si>
     <t>Associate software Developer</t>
+  </si>
+  <si>
+    <t>Conveyance</t>
+  </si>
+  <si>
+    <t>Fixed_Bonus</t>
+  </si>
+  <si>
+    <t>Performance_Bonus</t>
+  </si>
+  <si>
+    <t>Leaves</t>
+  </si>
+  <si>
+    <t>Provident_Fund</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Professional_Tax </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TDS_IT </t>
+  </si>
+  <si>
+    <t>Basic_DA</t>
+  </si>
+  <si>
+    <t>Pan_Card_Number</t>
+  </si>
+  <si>
+    <t>Total_Addition</t>
+  </si>
+  <si>
+    <t>Total_Deductions</t>
+  </si>
+  <si>
+    <t>Net_Salary</t>
+  </si>
+  <si>
+    <t>Payment_Mode</t>
+  </si>
+  <si>
+    <t>From_Bank_Name</t>
+  </si>
+  <si>
+    <t>Payment_Date</t>
+  </si>
+  <si>
+    <t>dfgyyy66666666767</t>
+  </si>
+  <si>
+    <t>NEFT</t>
+  </si>
+  <si>
+    <t>HDFC</t>
+  </si>
+  <si>
+    <t>shubham</t>
+  </si>
+  <si>
+    <t>shubhamj@lanatussystems.com</t>
+  </si>
+  <si>
+    <t>Special_Allowances</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,16 +163,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCFE2F3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -132,16 +192,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -423,110 +510,209 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:AC3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="33" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="20.85546875" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" customWidth="1"/>
+    <col min="9" max="9" width="26.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20.5703125" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" customWidth="1"/>
+    <col min="12" max="12" width="31.5703125" customWidth="1"/>
+    <col min="13" max="13" width="20.5703125" customWidth="1"/>
+    <col min="15" max="20" width="20.5703125" customWidth="1"/>
+    <col min="22" max="22" width="17.5703125" customWidth="1"/>
+    <col min="23" max="23" width="19" customWidth="1"/>
+    <col min="25" max="25" width="16.28515625" customWidth="1"/>
+    <col min="26" max="26" width="15.42578125" customWidth="1"/>
+    <col min="27" max="27" width="16.42578125" customWidth="1"/>
+    <col min="28" max="28" width="19" customWidth="1"/>
+    <col min="29" max="29" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="M1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" t="s">
+        <v>5</v>
+      </c>
+      <c r="O1" t="s">
         <v>15</v>
       </c>
-      <c r="I1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" t="s">
-        <v>17</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>18</v>
       </c>
-      <c r="M1" t="s">
-        <v>5</v>
-      </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
+        <v>38</v>
+      </c>
+      <c r="R1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O1" t="s">
+      <c r="S1" s="5" t="s">
         <v>20</v>
       </c>
+      <c r="T1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" t="s">
+        <v>21</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y1" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z1" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA1" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC1" s="6" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2">
+        <v>566655665</v>
+      </c>
+      <c r="H2">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2">
-        <v>566655665</v>
-      </c>
-      <c r="G2">
-        <v>6</v>
-      </c>
-      <c r="H2">
+      <c r="I2">
         <v>1</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>5</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="3">
+      <c r="L2" s="3">
         <v>44743</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>6000</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>2400</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>1600</v>
       </c>
-      <c r="O2">
-        <v>10000</v>
+      <c r="P2">
+        <v>5000</v>
+      </c>
+      <c r="Q2">
+        <v>5000</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>20000</v>
+      </c>
+      <c r="U2">
+        <v>300</v>
+      </c>
+      <c r="V2">
+        <v>1200</v>
+      </c>
+      <c r="W2">
+        <v>100</v>
+      </c>
+      <c r="X2">
+        <v>100</v>
+      </c>
+      <c r="Y2">
+        <v>1700</v>
+      </c>
+      <c r="Z2">
+        <v>18300</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC2" s="2">
+        <v>44984</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -534,43 +720,85 @@
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="2">
-        <v>44692</v>
-      </c>
-      <c r="F3">
-        <v>6465566</v>
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
       </c>
       <c r="G3">
+        <v>566655665</v>
+      </c>
+      <c r="H3">
         <v>6</v>
       </c>
-      <c r="H3">
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3" t="s">
+        <v>4</v>
+      </c>
+      <c r="L3" s="3">
+        <v>44743</v>
+      </c>
+      <c r="M3">
+        <v>6000</v>
+      </c>
+      <c r="N3">
+        <v>2400</v>
+      </c>
+      <c r="O3">
+        <v>1600</v>
+      </c>
+      <c r="P3">
+        <v>5000</v>
+      </c>
+      <c r="Q3">
+        <v>5000</v>
+      </c>
+      <c r="R3">
         <v>0</v>
       </c>
-      <c r="I3">
-        <v>6</v>
-      </c>
-      <c r="J3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K3" s="3">
-        <v>44774</v>
-      </c>
-      <c r="L3">
-        <v>7000</v>
-      </c>
-      <c r="M3">
-        <v>1000</v>
-      </c>
-      <c r="N3">
-        <v>2000</v>
-      </c>
-      <c r="O3">
-        <v>10000</v>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>20000</v>
+      </c>
+      <c r="U3">
+        <v>300</v>
+      </c>
+      <c r="V3">
+        <v>1200</v>
+      </c>
+      <c r="W3">
+        <v>100</v>
+      </c>
+      <c r="X3">
+        <v>100</v>
+      </c>
+      <c r="Y3">
+        <v>1700</v>
+      </c>
+      <c r="Z3">
+        <v>18300</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC3" s="2">
+        <v>44984</v>
       </c>
     </row>
   </sheetData>

</xml_diff>